<commit_message>
Update verified business reports
</commit_message>
<xml_diff>
--- a/reports/bulk_verification.xlsx
+++ b/reports/bulk_verification.xlsx
@@ -470,7 +470,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -519,7 +519,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>+919116135091</t>
+          <t>+91 91161 35108</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -626,11 +626,11 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>REVIEW REQUIRED</t>
+          <t>STRONG WEB SUPPORT</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -649,12 +649,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Multiple web sources were found, but at least one important field differs between sources. The conflicting field should be reviewed before treating the information as fully verified.</t>
+          <t>Multiple independent web sources provide supporting evidence with no major extracted-field conflict detected.</t>
         </is>
       </c>
     </row>
@@ -746,11 +746,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>REVIEW REQUIRED</t>
+          <t>STRONG WEB SUPPORT</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -759,7 +759,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>+91 99290 99748</t>
+          <t>+91 94140 71922</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -769,12 +769,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Multiple web sources were found, but at least one important field differs between sources. The conflicting field should be reviewed before treating the information as fully verified.</t>
+          <t>Multiple independent web sources provide supporting evidence with no major extracted-field conflict detected.</t>
         </is>
       </c>
     </row>
@@ -794,17 +794,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Laxmi Mishthan Bhandar, No</t>
+          <t>100-101, Johri Bazar, Bapu Bazar, Biseswarji, Jaipur, Rajasthan, 302003</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>+91 90246 09609</t>
+          <t>+91 9024609609</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Not found in current evidence</t>
+          <t>8 AM to 11 AM</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -826,35 +826,35 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>REVIEW REQUIRED</t>
+          <t>STRONG WEB SUPPORT</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2, Gandhi Path W, Acharya Vinoba Bhave Nagar, B Block, Vaishali Nagar, Jaipur</t>
+          <t>Not confidently extracted</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>+91 86969 17580</t>
+          <t>+918696917580</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>08:00 AM - 10:30 PM</t>
+          <t>Closed ⋅ Opens 11AM Phone: 090244 47555</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Multiple web sources were found, but at least one important field differs between sources. The conflicting field should be reviewed before treating the information as fully verified.</t>
+          <t>Multiple independent web sources provide supporting evidence with no major extracted-field conflict detected.</t>
         </is>
       </c>
     </row>
@@ -906,11 +906,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>STRONG WEB SUPPORT</t>
+          <t>REVIEW REQUIRED</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -929,12 +929,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Multiple independent web sources provide supporting evidence with no major extracted-field conflict detected.</t>
+          <t>Multiple web sources were found, but at least one important field differs between sources. The conflicting field should be reviewed before treating the information as fully verified.</t>
         </is>
       </c>
     </row>
@@ -986,20 +986,20 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>STRONG WEB SUPPORT</t>
+          <t>REVIEW REQUIRED</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Station Road Jaipur</t>
+          <t>Rawat Public School Sector-17, Pratap Nagar, Sanganer Jaipur (Rajasthan)-302033 Email: rawatpublicschool100@gmail.com narendra702@gmail.com Call: 0141-2796929, +91 7300000875, +91 8058007777 ## Useful</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Not found in current evidence</t>
+          <t>+91 7300000875</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1009,12 +1009,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Multiple independent web sources provide supporting evidence with no major extracted-field conflict detected.</t>
+          <t>Multiple web sources were found, but at least one important field differs between sources. The conflicting field should be reviewed before treating the information as fully verified.</t>
         </is>
       </c>
     </row>
@@ -1034,7 +1034,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>107,108 AJMERA GARDEN, SAMRAT, KINGS ROAD, AJMER ROAD, Jaipur</t>
+          <t>Not confidently extracted</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1066,20 +1066,20 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>REVIEW REQUIRED</t>
+          <t>STRONG WEB SUPPORT</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Janta Store Shopping Centre, University Marg, Bapu Nagar, Jaipur, Rajasthan 302015 Google Map: Ph: 089528 93657 Pricing: Tandoori Pizza: Rs</t>
+          <t>Not confidently extracted</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>+918949778386</t>
+          <t>+919664026168</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1089,12 +1089,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Multiple web sources were found, but at least one important field differs between sources. The conflicting field should be reviewed before treating the information as fully verified.</t>
+          <t>Multiple independent web sources provide supporting evidence with no major extracted-field conflict detected.</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Not confidently extracted</t>
+          <t>Hotel Clarks Amer, Jawahar Lal Nehru Marg, Jaipur 302017 CONTACT:EMAIL | PHONE CUISINE:Multi-cuisine TabluPhoto courtesy: Hotel Clarks Amer HappyTrips Editors TABLU - Hotel Clarks Amer Jaipur, Jaipur.</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1199,7 +1199,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>141-3610101</t>
+          <t>Not found in current evidence</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1226,20 +1226,20 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>REVIEW REQUIRED</t>
+          <t>STRONG WEB SUPPORT</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>(/cdn-cgi/l/email-protection)</t>
+          <t>Not confidently extracted</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>+919810372000</t>
+          <t>+919829166866</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1249,12 +1249,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Multiple web sources were found, but at least one important field differs between sources. The conflicting field should be reviewed before treating the information as fully verified.</t>
+          <t>Multiple independent web sources provide supporting evidence with no major extracted-field conflict detected.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update final verification reports
</commit_message>
<xml_diff>
--- a/reports/bulk_verification.xlsx
+++ b/reports/bulk_verification.xlsx
@@ -626,11 +626,11 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>STRONG WEB SUPPORT</t>
+          <t>REVIEW REQUIRED</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -649,12 +649,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Multiple independent web sources provide supporting evidence with no major extracted-field conflict detected.</t>
+          <t>Multiple web sources were found, but at least one important field differs between sources. The conflicting field should be reviewed before treating the information as fully verified.</t>
         </is>
       </c>
     </row>
@@ -794,17 +794,17 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>100-101, Johri Bazar, Bapu Bazar, Biseswarji, Jaipur, Rajasthan, 302003</t>
+          <t>Laxmi Mishthan Bhandar, No. 98, 99, Johari Bazar Rd, Bapu Bazar, Biseswarji, Jaipur, Rajasthan 302 003; tel: +91 90246 09609</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>+91 9024609609</t>
+          <t>+91 90246 09609</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>8 AM to 11 AM</t>
+          <t>Not found in current evidence</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Closed ⋅ Opens 11AM Phone: 090244 47555</t>
+          <t>Closed ⋅ Opens 11AM Phone: 090244 47555 Mahaveer Rabri Bhandar</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -884,7 +884,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>12:00 PM to 10:00 PM</t>
+          <t>Not found in current evidence</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -906,11 +906,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>REVIEW REQUIRED</t>
+          <t>STRONG WEB SUPPORT</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -929,12 +929,12 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Multiple web sources were found, but at least one important field differs between sources. The conflicting field should be reviewed before treating the information as fully verified.</t>
+          <t>Multiple independent web sources provide supporting evidence with no major extracted-field conflict detected.</t>
         </is>
       </c>
     </row>
@@ -986,20 +986,20 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>REVIEW REQUIRED</t>
+          <t>STRONG WEB SUPPORT</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>55</v>
+        <v>75</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Rawat Public School Sector-17, Pratap Nagar, Sanganer Jaipur (Rajasthan)-302033 Email: rawatpublicschool100@gmail.com narendra702@gmail.com Call: 0141-2796929, +91 7300000875, +91 8058007777 ## Useful</t>
+          <t>Tonk Road Jaipur</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>+91 7300000875</t>
+          <t>Not found in current evidence</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1009,12 +1009,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Multiple web sources were found, but at least one important field differs between sources. The conflicting field should be reviewed before treating the information as fully verified.</t>
+          <t>Multiple independent web sources provide supporting evidence with no major extracted-field conflict detected.</t>
         </is>
       </c>
     </row>
@@ -1066,11 +1066,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>STRONG WEB SUPPORT</t>
+          <t>REVIEW REQUIRED</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -1079,7 +1079,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>+919664026168</t>
+          <t>+918949778386</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1089,12 +1089,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Multiple independent web sources provide supporting evidence with no major extracted-field conflict detected.</t>
+          <t>Multiple web sources were found, but at least one important field differs between sources. The conflicting field should be reviewed before treating the information as fully verified.</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1199,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Not found in current evidence</t>
+          <t>141-3610101</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">

</xml_diff>

<commit_message>
Update bulk verification results
</commit_message>
<xml_diff>
--- a/reports/bulk_verification.xlsx
+++ b/reports/bulk_verification.xlsx
@@ -470,7 +470,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -514,7 +514,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Not confidently extracted</t>
+          <t>Ajmer Road, Jaipur, Rajasthan</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -626,11 +626,11 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>REVIEW REQUIRED</t>
+          <t>STRONG WEB SUPPORT</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>65</v>
+        <v>75</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -649,12 +649,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Multiple web sources were found, but at least one important field differs between sources. The conflicting field should be reviewed before treating the information as fully verified.</t>
+          <t>Multiple independent web sources provide supporting evidence with no major extracted-field conflict detected.</t>
         </is>
       </c>
     </row>
@@ -994,12 +994,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Tonk Road Jaipur</t>
+          <t>Not confidently extracted</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Not found in current evidence</t>
+          <t>0141-2170883</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Not confidently extracted</t>
+          <t>Janta Store Shopping Centre, University Marg, Bapu Nagar, Jaipur, Rajasthan 302015 Google Map: Ph: 089528 93657 Pricing: Tandoori Pizza: Rs.260 Egg Halwa: Rs.100 Watch Our Other Street Food Tours Mumb</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1114,7 +1114,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Not confidently extracted</t>
+          <t>Malviya Nagar Jaipur</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">

</xml_diff>